<commit_message>
bolsos + cambio en Back
</commit_message>
<xml_diff>
--- a/catalog/products.xlsx
+++ b/catalog/products.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAC6BE1-9BFB-482B-B396-EB7C63316E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E11ED1-F671-4521-9DAC-171C672F6136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="264">
   <si>
     <t>id</t>
   </si>
@@ -423,6 +423,390 @@
   </si>
   <si>
     <t>PSTK41000</t>
+  </si>
+  <si>
+    <t>BSTHEB51000</t>
+  </si>
+  <si>
+    <t>Paletero Hard Eva Black</t>
+  </si>
+  <si>
+    <t>bolso</t>
+  </si>
+  <si>
+    <t>paletero</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT04.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT06.png</t>
+  </si>
+  <si>
+    <t>hard eva eternal</t>
+  </si>
+  <si>
+    <t>BSTETE51000</t>
+  </si>
+  <si>
+    <t>Paletero Hard Eva Eternal</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT03.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT04.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT06.png</t>
+  </si>
+  <si>
+    <t>BSTONE51000</t>
+  </si>
+  <si>
+    <t>Paletero T-One Pro</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT03.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT04.png</t>
+  </si>
+  <si>
+    <t>BSTPM51000</t>
+  </si>
+  <si>
+    <t>Paletero Pro Master</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT05.png</t>
+  </si>
+  <si>
+    <t>pro master</t>
+  </si>
+  <si>
+    <t>star</t>
+  </si>
+  <si>
+    <t>BSTSTAR51000</t>
+  </si>
+  <si>
+    <t>Paletero Star</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT04.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT05.png</t>
+  </si>
+  <si>
+    <t>neon strike</t>
+  </si>
+  <si>
+    <t>BSTNEON51000</t>
+  </si>
+  <si>
+    <t>Paletero Neon Strike</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT03.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT04.png</t>
+  </si>
+  <si>
+    <t>m hard eva black</t>
+  </si>
+  <si>
+    <t>MSTHEB51000</t>
+  </si>
+  <si>
+    <t>Mochila Hard Eva Black</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT03.png</t>
+  </si>
+  <si>
+    <t>artic sport</t>
+  </si>
+  <si>
+    <t>MSTAR51000</t>
+  </si>
+  <si>
+    <t>Mochila Artic Sport</t>
+  </si>
+  <si>
+    <t>mochila</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT03.png</t>
+  </si>
+  <si>
+    <t>black voltage</t>
+  </si>
+  <si>
+    <t>MSTBV51000</t>
+  </si>
+  <si>
+    <t>Mochila Black Voltage</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT03.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT04.png</t>
+  </si>
+  <si>
+    <t>neceser navy</t>
+  </si>
+  <si>
+    <t>NSTNAVY51000</t>
+  </si>
+  <si>
+    <t>Neceser Navy</t>
+  </si>
+  <si>
+    <t>neceser</t>
+  </si>
+  <si>
+    <t>accesorio</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT03.png</t>
+  </si>
+  <si>
+    <t>neceser moss</t>
+  </si>
+  <si>
+    <t>NSTMOSS51000</t>
+  </si>
+  <si>
+    <t>Neceser Moss</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.MAIN.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT01.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT02.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT03.png</t>
+  </si>
+  <si>
+    <t>black cap</t>
+  </si>
+  <si>
+    <t>Black Cap</t>
+  </si>
+  <si>
+    <t>cap</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 4.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 2.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 1.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 3.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 5.png</t>
+  </si>
+  <si>
+    <t>power balance</t>
+  </si>
+  <si>
+    <t>Power Balance</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/POWER BALANCE.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/POWER BALANCE 2.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/ETERNAL1.5.webp</t>
+  </si>
+  <si>
+    <t>overgrip</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/OVERGRIP 60 UNITS 1.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/OVERGRIP 60 UNITS 3.png</t>
+  </si>
+  <si>
+    <t>Overgrip Premier Soft</t>
+  </si>
+  <si>
+    <t>Overgrip Tacky Touch</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/OVERGRIP 25 UNITS 1.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/OVERGRIP 25 UNITS 2.png</t>
+  </si>
+  <si>
+    <t>WristBand White</t>
+  </si>
+  <si>
+    <t>muniequera</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Muñequera blanca 4.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Muñequera blanca 1.png</t>
+  </si>
+  <si>
+    <t>Wristband Blue</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/MUÑEQUERA AZUL 1.1.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/MUÑEQUERA AZUL 1.2.png</t>
+  </si>
+  <si>
+    <t>Wristband Black x2</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Muñequera negra pack 2 2.png</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Muñequera negra pack 2 3.png</t>
+  </si>
+  <si>
+    <t>protector</t>
+  </si>
+  <si>
+    <t>Protector Transparent Carbon</t>
+  </si>
+  <si>
+    <t>key ring</t>
+  </si>
+  <si>
+    <t>Key Ring</t>
+  </si>
+  <si>
+    <t>llavero</t>
+  </si>
+  <si>
+    <t>t-one pro</t>
+  </si>
+  <si>
+    <t>hard eva black bag</t>
+  </si>
+  <si>
+    <t>overgrip premier soft</t>
+  </si>
+  <si>
+    <t>overgrip tacky touch</t>
+  </si>
+  <si>
+    <t>muñequera Wristband white</t>
+  </si>
+  <si>
+    <t>muñequera Wristband blue</t>
+  </si>
+  <si>
+    <t>muñequera Wristband black x2</t>
+  </si>
+  <si>
+    <t>protector transparent carbon</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/protector-transparente-carbono.webp</t>
   </si>
 </sst>
 </file>
@@ -805,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="19" width="22" customWidth="1"/>
@@ -887,7 +1271,7 @@
         <v>21</v>
       </c>
       <c r="F2">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
@@ -943,7 +1327,7 @@
         <v>21</v>
       </c>
       <c r="F3">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
@@ -1002,7 +1386,7 @@
         <v>21</v>
       </c>
       <c r="F4">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
@@ -1058,7 +1442,7 @@
         <v>21</v>
       </c>
       <c r="F5">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
@@ -1114,7 +1498,7 @@
         <v>66</v>
       </c>
       <c r="F6">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -1173,7 +1557,7 @@
         <v>66</v>
       </c>
       <c r="F7">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
@@ -1229,7 +1613,7 @@
         <v>83</v>
       </c>
       <c r="F8">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
@@ -1288,7 +1672,7 @@
         <v>83</v>
       </c>
       <c r="F9">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -1347,7 +1731,7 @@
         <v>83</v>
       </c>
       <c r="F10">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -1403,7 +1787,7 @@
         <v>83</v>
       </c>
       <c r="F11">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G11" t="b">
         <v>1</v>
@@ -1462,7 +1846,7 @@
         <v>122</v>
       </c>
       <c r="F12">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
@@ -1515,7 +1899,7 @@
         <v>122</v>
       </c>
       <c r="F13">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
@@ -1549,6 +1933,691 @@
       </c>
       <c r="S13">
         <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>256</v>
+      </c>
+      <c r="B14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" t="s">
+        <v>141</v>
+      </c>
+      <c r="J14" t="s">
+        <v>142</v>
+      </c>
+      <c r="K14" t="s">
+        <v>143</v>
+      </c>
+      <c r="S14">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>144</v>
+      </c>
+      <c r="B15" t="s">
+        <v>145</v>
+      </c>
+      <c r="C15" t="s">
+        <v>146</v>
+      </c>
+      <c r="D15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="s">
+        <v>147</v>
+      </c>
+      <c r="I15" t="s">
+        <v>148</v>
+      </c>
+      <c r="J15" t="s">
+        <v>149</v>
+      </c>
+      <c r="K15" t="s">
+        <v>150</v>
+      </c>
+      <c r="L15" t="s">
+        <v>151</v>
+      </c>
+      <c r="S15">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>255</v>
+      </c>
+      <c r="B16" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" t="s">
+        <v>153</v>
+      </c>
+      <c r="D16" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" t="s">
+        <v>139</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="s">
+        <v>154</v>
+      </c>
+      <c r="I16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J16" t="s">
+        <v>156</v>
+      </c>
+      <c r="K16" t="s">
+        <v>157</v>
+      </c>
+      <c r="L16" t="s">
+        <v>158</v>
+      </c>
+      <c r="S16">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" t="s">
+        <v>159</v>
+      </c>
+      <c r="C17" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" t="s">
+        <v>138</v>
+      </c>
+      <c r="E17" t="s">
+        <v>139</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="s">
+        <v>161</v>
+      </c>
+      <c r="I17" t="s">
+        <v>162</v>
+      </c>
+      <c r="J17" t="s">
+        <v>163</v>
+      </c>
+      <c r="K17" t="s">
+        <v>164</v>
+      </c>
+      <c r="S17">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C18" t="s">
+        <v>168</v>
+      </c>
+      <c r="D18" t="s">
+        <v>138</v>
+      </c>
+      <c r="E18" t="s">
+        <v>139</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="s">
+        <v>169</v>
+      </c>
+      <c r="I18" t="s">
+        <v>170</v>
+      </c>
+      <c r="J18" t="s">
+        <v>171</v>
+      </c>
+      <c r="K18" t="s">
+        <v>172</v>
+      </c>
+      <c r="L18" t="s">
+        <v>173</v>
+      </c>
+      <c r="S18">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>174</v>
+      </c>
+      <c r="B19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D19" t="s">
+        <v>138</v>
+      </c>
+      <c r="E19" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="s">
+        <v>177</v>
+      </c>
+      <c r="I19" t="s">
+        <v>178</v>
+      </c>
+      <c r="J19" t="s">
+        <v>179</v>
+      </c>
+      <c r="K19" t="s">
+        <v>180</v>
+      </c>
+      <c r="S19">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>181</v>
+      </c>
+      <c r="B20" t="s">
+        <v>182</v>
+      </c>
+      <c r="C20" t="s">
+        <v>183</v>
+      </c>
+      <c r="D20" t="s">
+        <v>191</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="s">
+        <v>184</v>
+      </c>
+      <c r="I20" t="s">
+        <v>185</v>
+      </c>
+      <c r="J20" t="s">
+        <v>186</v>
+      </c>
+      <c r="K20" t="s">
+        <v>187</v>
+      </c>
+      <c r="S20">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>188</v>
+      </c>
+      <c r="B21" t="s">
+        <v>189</v>
+      </c>
+      <c r="C21" t="s">
+        <v>190</v>
+      </c>
+      <c r="D21" t="s">
+        <v>191</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="s">
+        <v>192</v>
+      </c>
+      <c r="I21" t="s">
+        <v>193</v>
+      </c>
+      <c r="J21" t="s">
+        <v>194</v>
+      </c>
+      <c r="K21" t="s">
+        <v>195</v>
+      </c>
+      <c r="S21">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>196</v>
+      </c>
+      <c r="B22" t="s">
+        <v>197</v>
+      </c>
+      <c r="C22" t="s">
+        <v>198</v>
+      </c>
+      <c r="D22" t="s">
+        <v>191</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" t="s">
+        <v>199</v>
+      </c>
+      <c r="I22" t="s">
+        <v>200</v>
+      </c>
+      <c r="J22" t="s">
+        <v>201</v>
+      </c>
+      <c r="K22" t="s">
+        <v>202</v>
+      </c>
+      <c r="L22" t="s">
+        <v>203</v>
+      </c>
+      <c r="S22">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B23" t="s">
+        <v>205</v>
+      </c>
+      <c r="C23" t="s">
+        <v>206</v>
+      </c>
+      <c r="D23" t="s">
+        <v>208</v>
+      </c>
+      <c r="E23" t="s">
+        <v>207</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" t="s">
+        <v>209</v>
+      </c>
+      <c r="I23" t="s">
+        <v>210</v>
+      </c>
+      <c r="J23" t="s">
+        <v>211</v>
+      </c>
+      <c r="K23" t="s">
+        <v>212</v>
+      </c>
+      <c r="S23">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>213</v>
+      </c>
+      <c r="B24" t="s">
+        <v>214</v>
+      </c>
+      <c r="C24" t="s">
+        <v>215</v>
+      </c>
+      <c r="D24" t="s">
+        <v>208</v>
+      </c>
+      <c r="E24" t="s">
+        <v>207</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" t="s">
+        <v>216</v>
+      </c>
+      <c r="I24" t="s">
+        <v>217</v>
+      </c>
+      <c r="J24" t="s">
+        <v>218</v>
+      </c>
+      <c r="K24" t="s">
+        <v>219</v>
+      </c>
+      <c r="S24">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>220</v>
+      </c>
+      <c r="C25" t="s">
+        <v>221</v>
+      </c>
+      <c r="D25" t="s">
+        <v>208</v>
+      </c>
+      <c r="E25" t="s">
+        <v>222</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" t="s">
+        <v>223</v>
+      </c>
+      <c r="I25" t="s">
+        <v>224</v>
+      </c>
+      <c r="J25" t="s">
+        <v>225</v>
+      </c>
+      <c r="K25" t="s">
+        <v>226</v>
+      </c>
+      <c r="L25" t="s">
+        <v>227</v>
+      </c>
+      <c r="S25">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>228</v>
+      </c>
+      <c r="C26" t="s">
+        <v>229</v>
+      </c>
+      <c r="D26" t="s">
+        <v>208</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" t="s">
+        <v>230</v>
+      </c>
+      <c r="I26" t="s">
+        <v>231</v>
+      </c>
+      <c r="J26" t="s">
+        <v>232</v>
+      </c>
+      <c r="S26">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>257</v>
+      </c>
+      <c r="C27" t="s">
+        <v>236</v>
+      </c>
+      <c r="D27" t="s">
+        <v>208</v>
+      </c>
+      <c r="E27" t="s">
+        <v>233</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" t="s">
+        <v>234</v>
+      </c>
+      <c r="I27" t="s">
+        <v>235</v>
+      </c>
+      <c r="S27">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>258</v>
+      </c>
+      <c r="C28" t="s">
+        <v>237</v>
+      </c>
+      <c r="D28" t="s">
+        <v>208</v>
+      </c>
+      <c r="E28" t="s">
+        <v>233</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" t="s">
+        <v>238</v>
+      </c>
+      <c r="I28" t="s">
+        <v>239</v>
+      </c>
+      <c r="S28">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>259</v>
+      </c>
+      <c r="C29" t="s">
+        <v>240</v>
+      </c>
+      <c r="D29" t="s">
+        <v>208</v>
+      </c>
+      <c r="E29" t="s">
+        <v>241</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" t="s">
+        <v>242</v>
+      </c>
+      <c r="I29" t="s">
+        <v>243</v>
+      </c>
+      <c r="S29">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>260</v>
+      </c>
+      <c r="C30" t="s">
+        <v>244</v>
+      </c>
+      <c r="D30" t="s">
+        <v>208</v>
+      </c>
+      <c r="E30" t="s">
+        <v>241</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" t="s">
+        <v>245</v>
+      </c>
+      <c r="I30" t="s">
+        <v>246</v>
+      </c>
+      <c r="S30">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>261</v>
+      </c>
+      <c r="C31" t="s">
+        <v>247</v>
+      </c>
+      <c r="D31" t="s">
+        <v>208</v>
+      </c>
+      <c r="E31" t="s">
+        <v>241</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" t="s">
+        <v>248</v>
+      </c>
+      <c r="I31" t="s">
+        <v>249</v>
+      </c>
+      <c r="S31">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>262</v>
+      </c>
+      <c r="C32" t="s">
+        <v>251</v>
+      </c>
+      <c r="D32" t="s">
+        <v>208</v>
+      </c>
+      <c r="E32" t="s">
+        <v>250</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" t="s">
+        <v>263</v>
+      </c>
+      <c r="S32">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>252</v>
+      </c>
+      <c r="C33" t="s">
+        <v>253</v>
+      </c>
+      <c r="D33" t="s">
+        <v>208</v>
+      </c>
+      <c r="E33" t="s">
+        <v>254</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: complete StarVie catalog redesign and optimize assets
</commit_message>
<xml_diff>
--- a/catalog/products.xlsx
+++ b/catalog/products.xlsx
@@ -437,16 +437,16 @@
     <t>paletero</t>
   </si>
   <si>
-    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT04.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT06.png</t>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT04.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroHardEvaBlack/PALETERO STARVIE HARD EVA BLACK.PT06.webp</t>
   </si>
   <si>
     <t>hard eva eternal</t>
@@ -458,19 +458,19 @@
     <t>Paletero Hard Eva Eternal</t>
   </si>
   <si>
-    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT03.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT04.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT06.png</t>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT03.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT04.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroEternal/PALETERO STARVIE HARD EVA ETERNAL.PT06.webp</t>
   </si>
   <si>
     <t>BSTONE51000</t>
@@ -479,19 +479,19 @@
     <t>Paletero T-One Pro</t>
   </si>
   <si>
-    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT03.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT04.png</t>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT03.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroTone/PALETERO STARVIE T-ONE PRO.PT04.webp</t>
   </si>
   <si>
     <t>BSTPM51000</t>
@@ -500,16 +500,16 @@
     <t>Paletero Pro Master</t>
   </si>
   <si>
-    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT05.png</t>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroPromaster/PALETERO STARVIE PRO MASTER.PT05.webp</t>
   </si>
   <si>
     <t>pro master</t>
@@ -524,19 +524,19 @@
     <t>Paletero Star</t>
   </si>
   <si>
-    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT04.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT05.png</t>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT04.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroStar/PALETERO STARVIE STAR.PT05.webp</t>
   </si>
   <si>
     <t>neon strike</t>
@@ -548,16 +548,16 @@
     <t>Paletero Neon Strike</t>
   </si>
   <si>
-    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT03.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT04.png</t>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT03.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/paleteroNeon/PALETERO STARVIE NEON STRIKE.PT04.webp</t>
   </si>
   <si>
     <t>m hard eva black</t>
@@ -569,16 +569,16 @@
     <t>Mochila Hard Eva Black</t>
   </si>
   <si>
-    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT03.png</t>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaHardEva/MOCHILA STARVIE HARD EVA BLACK.PT03.webp</t>
   </si>
   <si>
     <t>artic sport</t>
@@ -593,16 +593,16 @@
     <t>mochila</t>
   </si>
   <si>
-    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT03.png</t>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaArtic/MOCHILA STARVIE ARTIC SPORT.PT03.webp</t>
   </si>
   <si>
     <t>black voltage</t>
@@ -614,16 +614,16 @@
     <t>Mochila Black Voltage</t>
   </si>
   <si>
-    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT03.png</t>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT03.webp</t>
   </si>
   <si>
     <t>products/bolsos/mochilaVoltage/MOCHILA STARVIE BLACK VOLTAGE.PT04.png</t>
@@ -644,16 +644,16 @@
     <t>accesorio</t>
   </si>
   <si>
-    <t>products/bolsos/neceser/NECESER STARVIE NAVY.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT03.png</t>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE NAVY.PT03.webp</t>
   </si>
   <si>
     <t>neceser moss</t>
@@ -665,16 +665,16 @@
     <t>Neceser Moss</t>
   </si>
   <si>
-    <t>products/bolsos/neceser/NECESER STARVIE MOSS.MAIN.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT01.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT02.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT03.png</t>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.MAIN.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT01.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT02.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/neceser/NECESER STARVIE MOSS.PT03.webp</t>
   </si>
   <si>
     <t>black cap</t>
@@ -686,19 +686,19 @@
     <t>cap</t>
   </si>
   <si>
-    <t>products/bolsos/accesorio/Gorra 4.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/accesorio/Gorra 2.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/accesorio/Gorra 1.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/accesorio/Gorra 3.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/accesorio/Gorra 5.png</t>
+    <t>products/bolsos/accesorio/Gorra 4.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 2.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 1.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 3.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Gorra 5.webp</t>
   </si>
   <si>
     <t>power balance</t>
@@ -743,10 +743,10 @@
     <t>muniequera</t>
   </si>
   <si>
-    <t>products/bolsos/accesorio/Muñequera blanca 4.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/accesorio/Muñequera blanca 1.png</t>
+    <t>products/bolsos/accesorio/Muñequera blanca 4.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Muñequera blanca 1.webp</t>
   </si>
   <si>
     <t>Wristband Blue</t>
@@ -761,10 +761,10 @@
     <t>Wristband Black x2</t>
   </si>
   <si>
-    <t>products/bolsos/accesorio/Muñequera negra pack 2 2.png</t>
-  </si>
-  <si>
-    <t>products/bolsos/accesorio/Muñequera negra pack 2 3.png</t>
+    <t>products/bolsos/accesorio/Muñequera negra pack 2 2.webp</t>
+  </si>
+  <si>
+    <t>products/bolsos/accesorio/Muñequera negra pack 2 3.webp</t>
   </si>
   <si>
     <t>protector</t>

</xml_diff>